<commit_message>
Sincronização Automática: 29/04/2026 10:13:47.72
</commit_message>
<xml_diff>
--- a/status.xlsx
+++ b/status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/miguel_santos_agrorobotica_com_br/Documents/AGROROBOTICA/PROJETOS/Dashboard_Retroagem_Laudos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="151" documentId="11_F25DC773A252ABDACC10489B791D7F6E5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF073CB4-D1C7-467B-8189-17C549887213}"/>
+  <xr:revisionPtr revIDLastSave="154" documentId="11_F25DC773A252ABDACC10489B791D7F6E5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{839E88A1-F0F1-41DF-9341-3E8EB2A01965}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -197,10 +197,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1042,7 +1038,7 @@
         <v>191</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1075,7 +1071,7 @@
         <v>193</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1108,7 +1104,7 @@
         <v>188</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sincronização Automática: 29/04/2026 11:37:57.09
</commit_message>
<xml_diff>
--- a/status.xlsx
+++ b/status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/miguel_santos_agrorobotica_com_br/Documents/AGROROBOTICA/PROJETOS/Dashboard_Retroagem_Laudos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="154" documentId="11_F25DC773A252ABDACC10489B791D7F6E5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{839E88A1-F0F1-41DF-9341-3E8EB2A01965}"/>
+  <xr:revisionPtr revIDLastSave="155" documentId="11_F25DC773A252ABDACC10489B791D7F6E5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FEFB760F-A417-4846-88A9-C840DB7068DE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -197,6 +197,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -994,7 +998,7 @@
         <v>200</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sincronização Automática: 29/04/2026 11:38:34.54
</commit_message>
<xml_diff>
--- a/status.xlsx
+++ b/status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/miguel_santos_agrorobotica_com_br/Documents/AGROROBOTICA/PROJETOS/Dashboard_Retroagem_Laudos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="155" documentId="11_F25DC773A252ABDACC10489B791D7F6E5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FEFB760F-A417-4846-88A9-C840DB7068DE}"/>
+  <xr:revisionPtr revIDLastSave="156" documentId="11_F25DC773A252ABDACC10489B791D7F6E5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{345833C0-7F88-482D-AB70-573278E91CA4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -998,7 +998,7 @@
         <v>200</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>